<commit_message>
Quota et tableau de bord séparés, régressions ok
</commit_message>
<xml_diff>
--- a/Cahier-de-recette-TOMSEN.xlsx
+++ b/Cahier-de-recette-TOMSEN.xlsx
@@ -3330,7 +3330,7 @@
       </c>
       <c r="E101" s="59" t="n"/>
     </row>
-    <row r="102" ht="36" customHeight="1">
+    <row r="102" ht="48.5" customHeight="1">
       <c r="A102" s="61" t="inlineStr">
         <is>
           <t>Cas 34</t>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="C102" s="63" t="inlineStr">
         <is>
-          <t>Préconditions : une récupération a été faite et 5 minutes se sont écoulées. Environnement de test de la Banque de France en réponse nominale.</t>
+          <t>Préconditions : une récupération a été faite et 5 minutes se sont écoulées. Environnement de test de la Banque de France en réponse nominale. Journal des requêtes fourni par Alice.</t>
         </is>
       </c>
       <c r="D102" s="63" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="D103" s="63" t="inlineStr">
         <is>
-          <t>La nouvelle demande est acceptée : les données et la date de mise à jour sont rafraîchies, sans message de quota</t>
+          <t>Le journal montre un nouvel appel vers banques/infos. Aucun message de quota ne s'affiche</t>
         </is>
       </c>
       <c r="E103" s="63" t="n"/>
@@ -3493,7 +3493,7 @@
       </c>
       <c r="D109" s="59" t="inlineStr">
         <is>
-          <t>Les blocs sont mis à jour et la date de dernière mise à jour change, sans message d'erreur</t>
+          <t>Les blocs de banque affichent les montants mis à jour. La date en bas de page change</t>
         </is>
       </c>
       <c r="E109" s="59" t="n"/>

</xml_diff>